<commit_message>
updated for w/c 14 Sept
updated Gantt and tracker, and hub
</commit_message>
<xml_diff>
--- a/files/Archive/Spinney_Gantt_v4.xlsx
+++ b/files/Archive/Spinney_Gantt_v4.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="274">
   <si>
     <t xml:space="preserve">Spinney External Works — Project Gantt (v4 — 3 Sep restructure: gate renumbering, render soft wash added, decking board-laying split from substructure)</t>
   </si>
@@ -192,7 +192,7 @@
     <t xml:space="preserve">2.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Decking side (a) — strip out, new substructure (incl. weed-stop membrane below). Investigate/replace leaking house waste pipe beneath chimney AND excavate to widen decking along side (a) — digger onsite from 3 Sep, this is today's work. Earth removed reused as buttress-wall infill along side (b). Widening is straight-line (distinct from the curved-decking-labour contingency purpose). Duration/cost partly unknown until pipe exposed — contingency-funded (likely purpose #9). Board-laying is now tracked separately at 2.5.</t>
+    <t xml:space="preserve">Decking side (a) — strip out, new substructure (incl. weed-stop membrane below). PIPE INVESTIGATION RESOLVED: no leaking waste pipe, damp ground was condensation under old decking. Excavation continues to widen decking, straight-line. Digger + barrow loader on hire until 10 Sep (est. £530, mixed purpose with new shed area — see 2.6). Earth reused as buttress-wall infill on side (b). RE-PLAN 8 Sep: all decking substructure (this + 2.3 + 2.6) now estimated to take 2 more weeks, ~22 Sep. Board-laying tracked separately at 2.5.</t>
   </si>
   <si>
     <t xml:space="preserve">In progress</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">2.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Decking side (b) — strip out, new substructure (incl. weed-stop membrane below). Old boards + substructure removed 17-18 Aug. Both lower and upper layer substructure under way (as of 3 Sep). Buttress walls infilled with earth excavated from side (a)'s dig (2.2). Travis Perkins order (F49820): ballast, sand, 72x solid dense blocks — TWO deliveries received, invoice still pending. Board-laying is now tracked separately at 2.5.</t>
+    <t xml:space="preserve">Decking side (b) — strip out, new substructure (incl. weed-stop membrane below). Old boards + substructure removed 17-18 Aug. Both lower and upper layer substructure under way. Buttress walls infilled with earth excavated from side (a)'s dig (2.2). Travis Perkins order (F49820): ballast, sand, 72x solid dense blocks — two deliveries received, invoice still pending. RE-PLAN 8 Sep: all decking substructure (this + 2.2 + 2.6) now estimated to take 2 more weeks, ~22 Sep. Board-laying tracked separately at 2.5.</t>
   </si>
   <si>
     <t xml:space="preserve">3.3</t>
@@ -225,13 +225,13 @@
     <t xml:space="preserve">2.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Lay Millboard decking per design, all sides (gate a and gate b access as applicable) — combined into one task for simplicity. Gated on G2 (gutters/slate) and G3 (tap/pipework/weed membrane).</t>
+    <t xml:space="preserve">Lay Millboard decking per design, all sides (gate a and gate b access as applicable) — INCLUDES the new decking area leading up to the shed, perpendicular to side (a). Combined into one task for simplicity. Gated on G2 (gutters/slate) and G3 (tap/pipework/weed membrane) AND substructure (2.2/2.3/2.6) completing. RE-PLAN 8 Sep: pushed back from 15 Sep — substructure now estimated to take 2 more weeks.</t>
   </si>
   <si>
     <t xml:space="preserve">G2, G3</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started (ESTIMATED — pushed back from 8 Sep placeholder since G2/G3 haven't started)</t>
+    <t xml:space="preserve">Not started (ESTIMATED, pushed back 8 Sep)</t>
   </si>
   <si>
     <t xml:space="preserve">G4</t>
@@ -246,7 +246,10 @@
     <t xml:space="preserve">2.6</t>
   </si>
   <si>
-    <t xml:space="preserve">Bonus — BBQ &amp; shed area from offcuts / excess, side (a)</t>
+    <t xml:space="preserve">New shed area, perpendicular to side (a) — TRIMMED 8 Sep to excavation + substructure only, for BOTH the shed base and the new decking area leading up to it. Millboard board-laying for that decking area is now tracked at 2.5 (gated on G2/G3). Shed relocation onto its own base is NOT dependent on board-laying — only on its own substructure — so it can happen as soon as substructure completes (~22 Sep), independent of G2/G3/2.5. RELATED to 3.3 (fence): boundary issue and scope increase, confirmed 8 Sep.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In progress — excavation phase, concurrent with 2.2/2.3</t>
   </si>
   <si>
     <t xml:space="preserve">G5</t>
@@ -273,12 +276,15 @@
     <t xml:space="preserve">Front-of-house gutters, minor roof repairs and tile repairs — repair / realignment (ladder work). Tile repairs confirmed via WhatsApp (10 Aug), same no-separate-charge basis.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fence spurring, side (b) — should complete before decking board-laying (2.5) starts; not blocking substructure work (2.3), which is already underway (propped temporarily).</t>
+    <t xml:space="preserve">Fence spurring, side (b) — should complete before decking board-laying (2.5) starts; not blocking substructure work (2.3), which is already under way (propped temporarily). UPDATE 8 Sep: repair/replacement, repositioned at new extended height — targeted by end of next week (w/c 14 Sep). RELATED to 2.6 (shed): boundary issue and scope increase confirmed 8 Sep — the two are connected, not independent.</t>
   </si>
   <si>
     <t xml:space="preserve">→ before 2.5</t>
   </si>
   <si>
+    <t xml:space="preserve">Propped temporarily — repair/reposition targeted end of w/c 14 Sep, new extended height</t>
+  </si>
+  <si>
     <t xml:space="preserve">3.4</t>
   </si>
   <si>
@@ -324,6 +330,24 @@
     <t xml:space="preserve">£141.66 est.</t>
   </si>
   <si>
+    <t xml:space="preserve">V4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V4 screw top-up #2 — 15 more boxes of Timberfix structural subframe screws (FH90P050), separate order from V3/purpose #8. Invoice received and PAID 10 Sep (£141.66, matching purpose #8 rate) — routed through Contingency (purpose #9), not this cost centre. Delivery scheduled 11 Sep.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid, delivery scheduled 11 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roofline works — gutter replacement (both parapet sides + lower rear elevation), fascia/soffit extension, slate replacement, barge board trim. NEW scope, own £2,140 budget. Estimate sent 4 Sep, discussed same day. Start confirmed 8 Sep: end of this week or next week (est.).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started (est.)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Non-working: Luke holiday w/c 27 Jul &amp; w/c 24 Aug (grey columns); UK bank holiday Mon 31 Aug (w/c 31 Aug is a 4-day week).</t>
   </si>
   <si>
@@ -495,7 +519,7 @@
     <t xml:space="preserve">Gate (a) ONLY</t>
   </si>
   <si>
-    <t xml:space="preserve">IN PROGRESS from 3 Sep — digger onsite. Earth reused as buttress-wall infill on side (b). Duration/cost partly unknown until pipe exposed — contingency-funded, likely purpose #9. Entrance = top-left of green deck on plan.</t>
+    <t xml:space="preserve">IN PROGRESS from 3 Sep. PIPE RESOLVED: no leak found — damp ground was condensation trapped under old decking, not a plumbing fault. No repair needed, no contingency draw required. Earth reused as buttress-wall infill on side (b). Entrance = top-left of green deck on plan.</t>
   </si>
   <si>
     <t xml:space="preserve">Decking (b)</t>
@@ -528,7 +552,7 @@
     <t xml:space="preserve">Decking (a+b)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lay Millboard decking per design, all sides — combined into one task for simplicity</t>
+    <t xml:space="preserve">Lay Millboard decking per design, all sides — combined into one task, including the new decking area leading up to the shed (perpendicular to side a)</t>
   </si>
   <si>
     <t xml:space="preserve">Gate (a) and gate (b) as applicable</t>
@@ -537,19 +561,19 @@
     <t xml:space="preserve">Gate a / Gate b</t>
   </si>
   <si>
-    <t xml:space="preserve">Gated on G2 (gutters/slate) and G3 (tap/pipework/weed membrane) clearing.</t>
+    <t xml:space="preserve">Gated on G2 (gutters/slate) and G3 (tap/pipework/weed membrane) clearing, plus substructure (2.2/2.3/2.6) completing.</t>
   </si>
   <si>
     <t xml:space="preserve">Decking (bonus)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lay offcuts / excess for new BBQ &amp; shed area</t>
+    <t xml:space="preserve">New shed area, perpendicular to side (a) — excavation + substructure only (shed base and the new decking area's substructure). Board-laying tracked separately at 2.5.</t>
   </si>
   <si>
     <t xml:space="preserve">Side (a)</t>
   </si>
   <si>
-    <t xml:space="preserve">Only when decking complete; uses surplus material.</t>
+    <t xml:space="preserve">RELATED to 3.3 (fence) — boundary issue and scope increase, confirmed 8 Sep. Shed relocation onto its own base is NOT gated by board-laying — only by this task's own substructure completing (~22 Sep).</t>
   </si>
   <si>
     <t xml:space="preserve">Driveway channel</t>
@@ -594,7 +618,7 @@
     <t xml:space="preserve">Garden</t>
   </si>
   <si>
-    <t xml:space="preserve">HARD CONSTRAINT (as designed): side (b) spurring should complete before decking board-laying (2.5) begins — access otherwise sub-optimal. STATUS 18 Aug: not yet done, but propped up temporarily and confirmed not to impact substructure laying. Deliberately deferred — Luke prefers wet weather for manipulating the fencing when actually fixing it. Rainy-day eligible, no fixed deadline pressure.</t>
+    <t xml:space="preserve">HARD CONSTRAINT (as designed): side (b) spurring should complete before decking board-laying (2.5) begins. STATUS 8 Sep: repair/replacement now confirmed, repositioned at new extended height, targeted by end of w/c 14 Sep. RELATED to 2.6 (shed) — boundary issue and scope increase, confirmed 8 Sep, the two are connected.</t>
   </si>
   <si>
     <t xml:space="preserve">Tree / bush clearing back to fence boundary — EXTERNAL company</t>
@@ -607,6 +631,18 @@
   </si>
   <si>
     <t xml:space="preserve">Gated on TPO decision (T1, date TBC). Both routes pre-planned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roofline works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gutter replacement (parapet both sides + lower rear), fascia/soffit extension, slate replacement, barge board trim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roofline, both sides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEW scope, own £2,140 budget. Estimate sent 4 Sep, discussed 4 Sep, start confirmed 8 Sep — end of this week or next. Distinct from earlier 'gutters included in Luke's price' understanding for 1.5/3.2 — confirm with Luke whether this supersedes or adds to that.</t>
   </si>
   <si>
     <t xml:space="preserve">Reference — contacts, rules, assumptions, sign-off log</t>
@@ -1440,7 +1476,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC42"/>
+  <dimension ref="A1:AC43"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -2188,7 +2224,9 @@
       <c r="G20" s="18" t="n">
         <v>46268</v>
       </c>
-      <c r="H20" s="18"/>
+      <c r="H20" s="18" t="n">
+        <v>46287</v>
+      </c>
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
       <c r="K20" s="15"/>
@@ -2233,7 +2271,9 @@
       <c r="G21" s="18" t="n">
         <v>46251</v>
       </c>
-      <c r="H21" s="18"/>
+      <c r="H21" s="18" t="n">
+        <v>46287</v>
+      </c>
       <c r="I21" s="14"/>
       <c r="J21" s="14"/>
       <c r="K21" s="15"/>
@@ -2368,10 +2408,10 @@
         <v>69</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
@@ -2413,10 +2453,10 @@
         <v>72</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="H25" s="19" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2434,42 +2474,42 @@
       </c>
       <c r="E26" s="16"/>
       <c r="F26" s="16" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G26" s="19" t="n">
-        <v>46310</v>
+        <v>46273</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>46314</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E27" s="16"/>
       <c r="F27" s="16" t="s">
         <v>72</v>
       </c>
       <c r="G27" s="19" t="n">
-        <v>46315</v>
+        <v>46323</v>
       </c>
       <c r="H27" s="19" t="n">
-        <v>46315</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -2502,10 +2542,10 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>15</v>
@@ -2545,10 +2585,10 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>15</v>
@@ -2591,19 +2631,19 @@
         <v>60</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E31" s="11" t="n">
         <v>3</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="G31" s="29"/>
       <c r="H31" s="29"/>
@@ -2631,13 +2671,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>16</v>
@@ -2646,7 +2686,7 @@
         <v>16</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G32" s="29"/>
       <c r="H32" s="29"/>
@@ -2674,16 +2714,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>15</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E33" s="11" t="n">
         <v>4</v>
@@ -2717,13 +2757,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="31" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B34" s="32" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D34" s="31" t="s">
         <v>53</v>
@@ -2758,13 +2798,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>16</v>
@@ -2801,10 +2841,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>52</v>
@@ -2813,39 +2853,86 @@
         <v>53</v>
       </c>
       <c r="E36" s="16" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F36" s="16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E37" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+    </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
-        <v>100</v>
+      <c r="A38" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="G38" s="19" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H38" s="19" t="n">
+        <v>46283</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>104</v>
+        <v>110</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>105</v>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2989,6 +3076,11 @@
       <formula>AND(ISNUMBER($G36),ISNUMBER($H36),$G36&lt;=I$5+6,$H36&gt;=I$5)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I38:AC38">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(ISNUMBER($G38),ISNUMBER($H38),$G38&lt;=I$5+6,$H38&gt;=I$5)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3004,7 +3096,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -3019,12 +3111,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3032,28 +3124,28 @@
         <v>4</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3061,28 +3153,28 @@
         <v>13</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H5" s="11" t="n">
         <v>2</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3090,28 +3182,28 @@
         <v>18</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H6" s="11" t="n">
         <v>2</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3119,28 +3211,28 @@
         <v>21</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C7" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>119</v>
       </c>
       <c r="H7" s="11" t="n">
         <v>7</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3148,28 +3240,28 @@
         <v>23</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C8" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="F8" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>124</v>
-      </c>
       <c r="G8" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>10</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3177,28 +3269,28 @@
         <v>25</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>1</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3206,28 +3298,28 @@
         <v>32</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H10" s="11" t="n">
         <v>3</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3235,28 +3327,28 @@
         <v>35</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>37</v>
       </c>
       <c r="I11" s="17" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3264,28 +3356,28 @@
         <v>44</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H12" s="11" t="n">
         <v>5</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3293,28 +3385,28 @@
         <v>55</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H13" s="16" t="n">
         <v>13</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3322,28 +3414,28 @@
         <v>58</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H14" s="16" t="n">
         <v>13</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3351,28 +3443,28 @@
         <v>61</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H15" s="16" t="s">
         <v>37</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3380,28 +3472,28 @@
         <v>66</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H16" s="16" t="n">
         <v>13</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3409,86 +3501,86 @@
         <v>73</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H17" s="11" t="n">
         <v>3</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H18" s="11" t="n">
         <v>4</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H19" s="11" t="n">
         <v>2</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3496,86 +3588,115 @@
         <v>60</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H20" s="11" t="n">
         <v>3</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H21" s="11" t="n">
         <v>2</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H22" s="11" t="n">
         <v>4</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>194</v>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="H23" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -3607,80 +3728,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="C5" s="36" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3688,68 +3809,68 @@
         <v>49</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E8" s="38" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="E9" s="37"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D10" s="37"/>
       <c r="E10" s="37"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D11" s="37"/>
       <c r="E11" s="37"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D12" s="37"/>
       <c r="E12" s="37"/>
@@ -3759,10 +3880,10 @@
         <v>20</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D13" s="37"/>
       <c r="E13" s="37"/>
@@ -3772,122 +3893,122 @@
         <v>52</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>52</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="E14" s="37"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="39" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="39" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="39" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="39" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="39" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="39" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="39" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="39" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="39" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="39" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="39" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="39" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="39" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="39" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>49</v>
@@ -3898,7 +4019,7 @@
         <v>27</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="C38" s="40" t="n">
         <v>46252</v>
@@ -3912,7 +4033,7 @@
         <v>39</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="C39" s="41"/>
       <c r="D39" s="41"/>
@@ -3924,7 +4045,7 @@
         <v>64</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="C40" s="41"/>
       <c r="D40" s="41"/>
@@ -3936,17 +4057,17 @@
         <v>70</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="C42" s="41"/>
       <c r="D42" s="41"/>
@@ -3956,42 +4077,42 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="39" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="39" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="39" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="39" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="39" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>